<commit_message>
Refactor: Framework cleanup and enhancements
- Removed @Parameters annotation; passed testID and inputID directly
- Added initializeTestContext() utility method
- Enhanced BasePage with interaction utilities and JavaDocs
- Updated testng.xml to align with new execution flow
- Cleaned config.properties for Excel and browser configs
</commit_message>
<xml_diff>
--- a/src/test/resources/POC_data_sheet_v1.1.xlsx
+++ b/src/test/resources/POC_data_sheet_v1.1.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SPidugujothi\IdeaProjects\AutomationPOC\src\test\resources\"/>
     </mc:Choice>
@@ -20,7 +20,7 @@
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="194">
   <si>
     <t>Application</t>
   </si>
@@ -591,12 +591,43 @@
   </si>
   <si>
     <t>13:46:42</t>
+  </si>
+  <si>
+    <t>R32</t>
+  </si>
+  <si>
+    <t>05/12/2025</t>
+  </si>
+  <si>
+    <t>23:42:03</t>
+  </si>
+  <si>
+    <t>R33</t>
+  </si>
+  <si>
+    <t>05/13/2025</t>
+  </si>
+  <si>
+    <t>00:24:19</t>
+  </si>
+  <si>
+    <t>element click intercepted: Element &lt;span class="cart-label"&gt;...&lt;/span&gt; is not clickable at point (10...</t>
+  </si>
+  <si>
+    <t>1987122</t>
+  </si>
+  <si>
+    <t>R34</t>
+  </si>
+  <si>
+    <t>00:26:49</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -672,7 +703,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -743,12 +774,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <top style="thin"/>
+    </border>
+    <border>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -835,6 +884,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="true">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="true"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1173,11 +1229,11 @@
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.44140625" style="17" customWidth="1"/>
-    <col min="2" max="2" width="31.44140625" customWidth="1"/>
-    <col min="3" max="3" width="21.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.109375" customWidth="1"/>
+    <col min="1" max="1" customWidth="true" style="17" width="8.44140625"/>
+    <col min="2" max="2" customWidth="true" width="31.44140625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="21.33203125"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="12.5546875"/>
+    <col min="6" max="6" customWidth="true" width="20.109375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.3">
@@ -1254,32 +1310,32 @@
   <dimension ref="A1:R5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="8.88671875" style="9"/>
-    <col min="3" max="3" width="13.5546875" style="9" customWidth="1"/>
-    <col min="4" max="4" width="26.21875" style="9" customWidth="1"/>
-    <col min="5" max="5" width="40.21875" style="9" customWidth="1"/>
-    <col min="6" max="6" width="7.44140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" style="9" customWidth="1"/>
-    <col min="8" max="8" width="12" style="9" customWidth="1"/>
-    <col min="9" max="9" width="29.21875" style="9" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.109375" style="9" customWidth="1"/>
-    <col min="12" max="12" width="7.6640625" style="9" customWidth="1"/>
-    <col min="13" max="13" width="15.77734375" style="9" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.109375" style="9" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20" style="9" customWidth="1"/>
-    <col min="16" max="16" width="7.6640625" style="9" customWidth="1"/>
-    <col min="17" max="17" width="12.77734375" style="9" customWidth="1"/>
-    <col min="18" max="18" width="11" style="9" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="12.77734375" style="9" customWidth="1"/>
-    <col min="20" max="20" width="8.88671875" style="9"/>
-    <col min="21" max="21" width="21.77734375" style="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.6640625" style="9" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.44140625" style="9" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.21875" style="9" customWidth="1"/>
-    <col min="25" max="25" width="12.5546875" style="9" customWidth="1"/>
-    <col min="26" max="16384" width="8.88671875" style="9"/>
+    <col min="1" max="1" customWidth="true" style="9" width="16.44140625"/>
+    <col min="2" max="2" style="9" width="8.88671875"/>
+    <col min="3" max="3" customWidth="true" style="9" width="13.5546875"/>
+    <col min="4" max="4" customWidth="true" style="9" width="26.21875"/>
+    <col min="5" max="5" customWidth="true" style="9" width="40.21875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" style="9" width="7.44140625"/>
+    <col min="7" max="7" customWidth="true" style="9" width="10.6640625"/>
+    <col min="8" max="8" customWidth="true" style="9" width="12.0"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" style="9" width="29.21875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" style="9" width="11.5546875"/>
+    <col min="11" max="11" customWidth="true" style="9" width="15.109375"/>
+    <col min="12" max="12" customWidth="true" style="9" width="7.6640625"/>
+    <col min="13" max="13" bestFit="true" customWidth="true" style="9" width="15.77734375"/>
+    <col min="14" max="14" bestFit="true" customWidth="true" style="9" width="15.109375"/>
+    <col min="15" max="15" customWidth="true" style="9" width="20.0"/>
+    <col min="16" max="16" customWidth="true" style="9" width="7.6640625"/>
+    <col min="17" max="17" customWidth="true" style="9" width="12.77734375"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" style="9" width="11.0"/>
+    <col min="19" max="19" customWidth="true" style="9" width="12.77734375"/>
+    <col min="20" max="20" style="9" width="8.88671875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" style="9" width="21.77734375"/>
+    <col min="22" max="22" bestFit="true" customWidth="true" style="9" width="13.6640625"/>
+    <col min="23" max="23" bestFit="true" customWidth="true" style="9" width="13.44140625"/>
+    <col min="24" max="24" customWidth="true" style="9" width="15.21875"/>
+    <col min="25" max="25" customWidth="true" style="9" width="12.5546875"/>
+    <col min="26" max="16384" style="9" width="8.88671875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="13" customFormat="1" x14ac:dyDescent="0.3">
@@ -1551,16 +1607,16 @@
   <dimension ref="A1:L54"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.5546875" customWidth="1"/>
-    <col min="6" max="6" width="6.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.5546875" customWidth="1"/>
-    <col min="8" max="9" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.44140625" customWidth="1"/>
-    <col min="11" max="11" width="11.88671875" customWidth="1"/>
-    <col min="12" max="12" width="50" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="12.5546875"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="12.88671875"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="25.77734375"/>
+    <col min="5" max="5" customWidth="true" width="36.5546875"/>
+    <col min="6" max="6" bestFit="true" customWidth="true" width="6.77734375"/>
+    <col min="7" max="7" customWidth="true" width="14.5546875"/>
+    <col min="8" max="9" bestFit="true" customWidth="true" width="14.88671875"/>
+    <col min="10" max="10" customWidth="true" width="10.44140625"/>
+    <col min="11" max="11" customWidth="true" width="11.88671875"/>
+    <col min="12" max="12" customWidth="true" width="50.0"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
@@ -2449,10 +2505,18 @@
       <c r="C34" s="20"/>
       <c r="D34" s="20"/>
       <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="20"/>
-      <c r="H34" s="20"/>
-      <c r="I34" s="20"/>
+      <c r="F34" t="s" s="32">
+        <v>184</v>
+      </c>
+      <c r="G34" t="s" s="32">
+        <v>185</v>
+      </c>
+      <c r="H34" t="s" s="32">
+        <v>186</v>
+      </c>
+      <c r="I34" t="s" s="32">
+        <v>78</v>
+      </c>
       <c r="J34" s="20"/>
       <c r="K34" s="20"/>
       <c r="L34" s="20"/>
@@ -2465,13 +2529,23 @@
       <c r="E35" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
-      <c r="H35" s="20"/>
-      <c r="I35" s="20"/>
+      <c r="F35" t="s" s="33">
+        <v>187</v>
+      </c>
+      <c r="G35" t="s" s="33">
+        <v>188</v>
+      </c>
+      <c r="H35" t="s" s="33">
+        <v>189</v>
+      </c>
+      <c r="I35" t="s" s="33">
+        <v>72</v>
+      </c>
       <c r="J35" s="20"/>
       <c r="K35" s="20"/>
-      <c r="L35" s="20"/>
+      <c r="L35" t="s" s="34">
+        <v>190</v>
+      </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="20"/>
@@ -2481,12 +2555,24 @@
       <c r="E36" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="F36" s="20"/>
-      <c r="G36" s="20"/>
-      <c r="H36" s="20"/>
-      <c r="I36" s="20"/>
-      <c r="J36" s="20"/>
-      <c r="K36" s="20"/>
+      <c r="F36" t="s" s="36">
+        <v>192</v>
+      </c>
+      <c r="G36" t="s" s="36">
+        <v>188</v>
+      </c>
+      <c r="H36" t="s" s="36">
+        <v>193</v>
+      </c>
+      <c r="I36" t="s" s="36">
+        <v>78</v>
+      </c>
+      <c r="J36" t="s" s="35">
+        <v>191</v>
+      </c>
+      <c r="K36" t="s" s="35">
+        <v>185</v>
+      </c>
       <c r="L36" s="20"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
@@ -2778,17 +2864,17 @@
   <dimension ref="A1:K4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.77734375" customWidth="1"/>
-    <col min="3" max="3" width="15.77734375" customWidth="1"/>
-    <col min="4" max="4" width="27.109375" customWidth="1"/>
-    <col min="5" max="5" width="34.77734375" customWidth="1"/>
-    <col min="6" max="6" width="13.5546875" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="10.44140625"/>
+    <col min="2" max="2" customWidth="true" width="16.77734375"/>
+    <col min="3" max="3" customWidth="true" width="15.77734375"/>
+    <col min="4" max="4" customWidth="true" width="27.109375"/>
+    <col min="5" max="5" customWidth="true" width="34.77734375"/>
+    <col min="6" max="6" customWidth="true" width="13.5546875"/>
+    <col min="7" max="7" bestFit="true" customWidth="true" width="13.44140625"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="13.6640625"/>
+    <col min="9" max="9" bestFit="true" customWidth="true" width="14.88671875"/>
+    <col min="10" max="10" bestFit="true" customWidth="true" width="7.6640625"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="9.77734375"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
feat(framework): E2E reorder + Jira/Excel/Email overhaul; cleaner pages/flows/base
Jira: rich ADF summary, inline screenshot (mediaId), create/search/update, local key store, attach report/screenshot w/ retry, add link to Extent, listener ensures single exec write.
Excel: execution data writer w/ next RunID (System/E2E), failure reason wrap; E2E Binding sync from Transactional with global dedupe; order data writer.
Email: SMTP sender w/ domain grouping, STARTTLS, env/Base64 creds, report attachment.
Pages/Flows: AddProducts..., Login, Register, OrderInformation + ReorderFlow; stronger waits, logging, small fixes.
Core: BaseTest lifecycle + screenshot-on-failure, context attrs; FileAwait; TestTypeUtil + @TestType.
Config/TestNG/POM updates; formatting/docs; keep 'no usages' items as requested.
</commit_message>
<xml_diff>
--- a/src/test/resources/POC_data_sheet_v1.1.xlsx
+++ b/src/test/resources/POC_data_sheet_v1.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SPidugujothi\IdeaProjects\MyridiusUAF\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33481A8C-BEDC-47BF-A1C4-E6BA37202D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA79DA60-A14B-4B13-975C-32EA904489EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="3" xr2:uid="{08B05D20-EDEF-43CA-A5DF-998FB408C439}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="963" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1152" uniqueCount="551">
   <si>
     <t>Application</t>
   </si>
@@ -1136,9 +1136,6 @@
     <t>Register Time</t>
   </si>
   <si>
-    <t>2025-07-27</t>
-  </si>
-  <si>
     <t>R102</t>
   </si>
   <si>
@@ -1235,42 +1232,6 @@
     <t>Expected condition failed: waiting for element to be clickable: Proxy element for: DefaultElementLoc…</t>
   </si>
   <si>
-    <t>21:26:32</t>
-  </si>
-  <si>
-    <t>21:28:24</t>
-  </si>
-  <si>
-    <t>21:31:25</t>
-  </si>
-  <si>
-    <t>2057437</t>
-  </si>
-  <si>
-    <t>21:45:26</t>
-  </si>
-  <si>
-    <t>2057446</t>
-  </si>
-  <si>
-    <t>22:08:39</t>
-  </si>
-  <si>
-    <t>amit.patel548@gmail.com</t>
-  </si>
-  <si>
-    <t>U7zBhiD7R0</t>
-  </si>
-  <si>
-    <t>22:18:39</t>
-  </si>
-  <si>
-    <t>2057456</t>
-  </si>
-  <si>
-    <t>22:20:24</t>
-  </si>
-  <si>
     <t>R115</t>
   </si>
   <si>
@@ -1349,27 +1310,9 @@
     <t>SC1-TC1-E2E-Reorder</t>
   </si>
   <si>
-    <t>divya.yadav453@yahoo.com</t>
-  </si>
-  <si>
-    <t>dLJv5nFgww</t>
-  </si>
-  <si>
-    <t>2025-07-30</t>
-  </si>
-  <si>
-    <t>16:28:36</t>
-  </si>
-  <si>
-    <t>2061022</t>
-  </si>
-  <si>
     <t>07/30/2025</t>
   </si>
   <si>
-    <t>16:30:53</t>
-  </si>
-  <si>
     <t>R126</t>
   </si>
   <si>
@@ -1382,25 +1325,376 @@
     <t>18:44:05</t>
   </si>
   <si>
-    <t>rohan.singh229@yahoo.com</t>
-  </si>
-  <si>
-    <t>*MAagSfDyI</t>
-  </si>
-  <si>
-    <t>18:56:09</t>
-  </si>
-  <si>
-    <t>2061138</t>
-  </si>
-  <si>
-    <t>18:58:31</t>
-  </si>
-  <si>
     <t>R128</t>
   </si>
   <si>
     <t>21:25:14</t>
+  </si>
+  <si>
+    <t>R129</t>
+  </si>
+  <si>
+    <t>08/01/2025</t>
+  </si>
+  <si>
+    <t>16:30:43</t>
+  </si>
+  <si>
+    <t>R130</t>
+  </si>
+  <si>
+    <t>20:33:10</t>
+  </si>
+  <si>
+    <t>R131</t>
+  </si>
+  <si>
+    <t>08/02/2025</t>
+  </si>
+  <si>
+    <t>08:28:31</t>
+  </si>
+  <si>
+    <t>R132</t>
+  </si>
+  <si>
+    <t>08:55:41</t>
+  </si>
+  <si>
+    <t>R133</t>
+  </si>
+  <si>
+    <t>09:02:58</t>
+  </si>
+  <si>
+    <t>Login was not successful for user: rohan.singh229@yahoo.com</t>
+  </si>
+  <si>
+    <t>R134</t>
+  </si>
+  <si>
+    <t>09:06:36</t>
+  </si>
+  <si>
+    <t>R135</t>
+  </si>
+  <si>
+    <t>09:14:54</t>
+  </si>
+  <si>
+    <t>R136</t>
+  </si>
+  <si>
+    <t>09:20:15</t>
+  </si>
+  <si>
+    <t>R137</t>
+  </si>
+  <si>
+    <t>10:54:01</t>
+  </si>
+  <si>
+    <t>R138</t>
+  </si>
+  <si>
+    <t>11:04:06</t>
+  </si>
+  <si>
+    <t>R139</t>
+  </si>
+  <si>
+    <t>11:11:54</t>
+  </si>
+  <si>
+    <t>R140</t>
+  </si>
+  <si>
+    <t>11:16:46</t>
+  </si>
+  <si>
+    <t>R141</t>
+  </si>
+  <si>
+    <t>11:22:58</t>
+  </si>
+  <si>
+    <t>R142</t>
+  </si>
+  <si>
+    <t>11:26:28</t>
+  </si>
+  <si>
+    <t>R143</t>
+  </si>
+  <si>
+    <t>08/09/2025</t>
+  </si>
+  <si>
+    <t>23:31:30</t>
+  </si>
+  <si>
+    <t>R144</t>
+  </si>
+  <si>
+    <t>23:41:47</t>
+  </si>
+  <si>
+    <t>R145</t>
+  </si>
+  <si>
+    <t>08/11/2025</t>
+  </si>
+  <si>
+    <t>11:31:36</t>
+  </si>
+  <si>
+    <t>R146</t>
+  </si>
+  <si>
+    <t>11:35:57</t>
+  </si>
+  <si>
+    <t>R147</t>
+  </si>
+  <si>
+    <t>11:46:15</t>
+  </si>
+  <si>
+    <t>R148</t>
+  </si>
+  <si>
+    <t>11:55:18</t>
+  </si>
+  <si>
+    <t>R149</t>
+  </si>
+  <si>
+    <t>12:02:17</t>
+  </si>
+  <si>
+    <t>R150</t>
+  </si>
+  <si>
+    <t>13:28:44</t>
+  </si>
+  <si>
+    <t>R151</t>
+  </si>
+  <si>
+    <t>13:28:53</t>
+  </si>
+  <si>
+    <t>The supplied file was empty (zero bytes long)</t>
+  </si>
+  <si>
+    <t>R152</t>
+  </si>
+  <si>
+    <t>16:09:39</t>
+  </si>
+  <si>
+    <t>R153</t>
+  </si>
+  <si>
+    <t>16:20:50</t>
+  </si>
+  <si>
+    <t>R154</t>
+  </si>
+  <si>
+    <t>16:30:44</t>
+  </si>
+  <si>
+    <t>R155</t>
+  </si>
+  <si>
+    <t>16:35:14</t>
+  </si>
+  <si>
+    <t>2025-08-11</t>
+  </si>
+  <si>
+    <t>R156</t>
+  </si>
+  <si>
+    <t>17:12:55</t>
+  </si>
+  <si>
+    <t>R157</t>
+  </si>
+  <si>
+    <t>17:43:14</t>
+  </si>
+  <si>
+    <t>R158</t>
+  </si>
+  <si>
+    <t>19:03:47</t>
+  </si>
+  <si>
+    <t>R159</t>
+  </si>
+  <si>
+    <t>19:10:51</t>
+  </si>
+  <si>
+    <t>R160</t>
+  </si>
+  <si>
+    <t>19:45:54</t>
+  </si>
+  <si>
+    <t>rahul.reddy917@outlook.com</t>
+  </si>
+  <si>
+    <t>kX6*KwD%cy</t>
+  </si>
+  <si>
+    <t>20:19:03</t>
+  </si>
+  <si>
+    <t>R161</t>
+  </si>
+  <si>
+    <t>20:19:25</t>
+  </si>
+  <si>
+    <t>R162</t>
+  </si>
+  <si>
+    <t>20:22:16</t>
+  </si>
+  <si>
+    <t>Invalid gender: Male89. Allowed: [male, female]</t>
+  </si>
+  <si>
+    <t>R163</t>
+  </si>
+  <si>
+    <t>08/12/2025</t>
+  </si>
+  <si>
+    <t>00:18:06</t>
+  </si>
+  <si>
+    <t>2077088</t>
+  </si>
+  <si>
+    <t>R164</t>
+  </si>
+  <si>
+    <t>09:56:12</t>
+  </si>
+  <si>
+    <t>R165</t>
+  </si>
+  <si>
+    <t>22:04:25</t>
+  </si>
+  <si>
+    <t>08/11/2026</t>
+  </si>
+  <si>
+    <t>R166</t>
+  </si>
+  <si>
+    <t>22:39:50</t>
+  </si>
+  <si>
+    <t>2077781</t>
+  </si>
+  <si>
+    <t>R167</t>
+  </si>
+  <si>
+    <t>22:40:50</t>
+  </si>
+  <si>
+    <t>R168</t>
+  </si>
+  <si>
+    <t>08/12/2026</t>
+  </si>
+  <si>
+    <t>22:40:51</t>
+  </si>
+  <si>
+    <t>R169</t>
+  </si>
+  <si>
+    <t>23:20:37</t>
+  </si>
+  <si>
+    <t>R170</t>
+  </si>
+  <si>
+    <t>23:24:56</t>
+  </si>
+  <si>
+    <t>2077792</t>
+  </si>
+  <si>
+    <t>E2E1</t>
+  </si>
+  <si>
+    <t>23:29:04</t>
+  </si>
+  <si>
+    <t>R171</t>
+  </si>
+  <si>
+    <t>08/13/2025</t>
+  </si>
+  <si>
+    <t>07:24:34</t>
+  </si>
+  <si>
+    <t>2077932</t>
+  </si>
+  <si>
+    <t>R172</t>
+  </si>
+  <si>
+    <t>07:40:21</t>
+  </si>
+  <si>
+    <t>2077943</t>
+  </si>
+  <si>
+    <t>E2E2</t>
+  </si>
+  <si>
+    <t>08:07:26</t>
+  </si>
+  <si>
+    <t>2077988</t>
+  </si>
+  <si>
+    <t>E2E3</t>
+  </si>
+  <si>
+    <t>09:07:32</t>
+  </si>
+  <si>
+    <t>E2E4</t>
+  </si>
+  <si>
+    <t>12:48:04</t>
+  </si>
+  <si>
+    <t>E2E5</t>
+  </si>
+  <si>
+    <t>12:48:28</t>
+  </si>
+  <si>
+    <t>No row found for key: Ip7 in sheet: Synthetic_Data (col 5)</t>
+  </si>
+  <si>
+    <t>E2E6</t>
+  </si>
+  <si>
+    <t>13:04:03</t>
   </si>
 </sst>
 </file>
@@ -1483,7 +1777,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -1716,6 +2010,139 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <top style="thin"/>
     </border>
     <border>
@@ -1738,7 +2165,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1842,13 +2269,30 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1869,18 +2313,13 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true">
       <alignment wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="true"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2261,11 +2700,11 @@
       <c r="B2" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C2" t="s" s="60">
-        <v>446</v>
-      </c>
-      <c r="D2" t="s" s="60">
-        <v>447</v>
+      <c r="C2" t="s" s="0">
+        <v>500</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>501</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>31</v>
@@ -2273,11 +2712,11 @@
       <c r="F2" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G2" t="s" s="60">
-        <v>437</v>
-      </c>
-      <c r="H2" t="s" s="60">
-        <v>448</v>
+      <c r="G2" t="s" s="0">
+        <v>489</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>502</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -2345,28 +2784,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="59" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="49" t="s">
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="G1" s="49"/>
-      <c r="H1" s="49"/>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
-      <c r="K1" s="49"/>
-      <c r="L1" s="49"/>
-      <c r="M1" s="49"/>
-      <c r="N1" s="49"/>
-      <c r="O1" s="49"/>
-      <c r="P1" s="49"/>
-      <c r="Q1" s="49"/>
-      <c r="R1" s="50"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
+      <c r="L1" s="60"/>
+      <c r="M1" s="60"/>
+      <c r="N1" s="60"/>
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="61"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
@@ -2610,7 +3049,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{087D34EC-64B6-464A-B1FA-1B3B12C5A42D}">
-  <dimension ref="A1:L130"/>
+  <dimension ref="A1:L179"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="15.44140625"/>
@@ -2628,23 +3067,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="62" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="52" t="s">
+      <c r="B1" s="62"/>
+      <c r="C1" s="62"/>
+      <c r="D1" s="62"/>
+      <c r="E1" s="62"/>
+      <c r="F1" s="63" t="s">
         <v>116</v>
       </c>
-      <c r="G1" s="52"/>
-      <c r="H1" s="52"/>
-      <c r="I1" s="52"/>
-      <c r="J1" s="53" t="s">
+      <c r="G1" s="63"/>
+      <c r="H1" s="63"/>
+      <c r="I1" s="63"/>
+      <c r="J1" s="64" t="s">
         <v>117</v>
       </c>
-      <c r="K1" s="53"/>
+      <c r="K1" s="64"/>
       <c r="L1" s="17"/>
     </row>
     <row r="2" spans="1:12" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -5217,13 +5656,13 @@
     </row>
     <row r="104" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F104" s="39" t="s">
+        <v>364</v>
+      </c>
+      <c r="G104" s="39" t="s">
         <v>365</v>
       </c>
-      <c r="G104" s="39" t="s">
+      <c r="H104" s="39" t="s">
         <v>366</v>
-      </c>
-      <c r="H104" s="39" t="s">
-        <v>367</v>
       </c>
       <c r="I104" s="39" t="s">
         <v>72</v>
@@ -5231,13 +5670,13 @@
     </row>
     <row r="105" spans="6:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="F105" s="39" t="s">
+        <v>367</v>
+      </c>
+      <c r="G105" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="H105" s="39" t="s">
         <v>368</v>
-      </c>
-      <c r="G105" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="H105" s="39" t="s">
-        <v>369</v>
       </c>
       <c r="I105" s="39" t="s">
         <v>66</v>
@@ -5248,30 +5687,30 @@
     </row>
     <row r="106" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F106" s="39" t="s">
+        <v>369</v>
+      </c>
+      <c r="G106" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="H106" s="39" t="s">
         <v>370</v>
       </c>
-      <c r="G106" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="H106" s="39" t="s">
+      <c r="I106" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="L106" s="40" t="s">
         <v>371</v>
-      </c>
-      <c r="I106" s="39" t="s">
-        <v>66</v>
-      </c>
-      <c r="L106" s="40" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="107" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F107" s="39" t="s">
+        <v>372</v>
+      </c>
+      <c r="G107" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="H107" s="39" t="s">
         <v>373</v>
-      </c>
-      <c r="G107" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="H107" s="39" t="s">
-        <v>374</v>
       </c>
       <c r="I107" s="39" t="s">
         <v>72</v>
@@ -5279,13 +5718,13 @@
     </row>
     <row r="108" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F108" s="39" t="s">
+        <v>374</v>
+      </c>
+      <c r="G108" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="H108" s="39" t="s">
         <v>375</v>
-      </c>
-      <c r="G108" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="H108" s="39" t="s">
-        <v>376</v>
       </c>
       <c r="I108" s="39" t="s">
         <v>72</v>
@@ -5293,13 +5732,13 @@
     </row>
     <row r="109" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F109" s="39" t="s">
+        <v>376</v>
+      </c>
+      <c r="G109" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="H109" s="39" t="s">
         <v>377</v>
-      </c>
-      <c r="G109" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="H109" s="39" t="s">
-        <v>378</v>
       </c>
       <c r="I109" s="39" t="s">
         <v>66</v>
@@ -5310,87 +5749,87 @@
     </row>
     <row r="110" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F110" s="39" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="G110" s="39" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="H110" s="39" t="s">
+        <v>378</v>
+      </c>
+      <c r="I110" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="L110" s="40" t="s">
         <v>379</v>
-      </c>
-      <c r="I110" s="39" t="s">
-        <v>66</v>
-      </c>
-      <c r="L110" s="40" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="111" spans="6:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="F111" s="39" t="s">
+        <v>380</v>
+      </c>
+      <c r="G111" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="H111" s="39" t="s">
         <v>381</v>
       </c>
-      <c r="G111" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="H111" s="39" t="s">
+      <c r="I111" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="L111" s="40" t="s">
         <v>382</v>
-      </c>
-      <c r="I111" s="39" t="s">
-        <v>66</v>
-      </c>
-      <c r="L111" s="40" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="112" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F112" s="39" t="s">
+        <v>383</v>
+      </c>
+      <c r="G112" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="H112" s="39" t="s">
         <v>384</v>
       </c>
-      <c r="G112" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="H112" s="39" t="s">
-        <v>385</v>
-      </c>
       <c r="I112" s="39" t="s">
         <v>66</v>
       </c>
       <c r="L112" s="40" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="113" spans="6:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="F113" s="39" t="s">
+        <v>385</v>
+      </c>
+      <c r="G113" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="H113" s="39" t="s">
         <v>386</v>
       </c>
-      <c r="G113" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="H113" s="39" t="s">
-        <v>387</v>
-      </c>
       <c r="I113" s="39" t="s">
         <v>66</v>
       </c>
       <c r="L113" s="40" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="114" spans="6:12" x14ac:dyDescent="0.3">
       <c r="F114" s="39" t="s">
+        <v>388</v>
+      </c>
+      <c r="G114" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="H114" s="39" t="s">
         <v>389</v>
       </c>
-      <c r="G114" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="H114" s="39" t="s">
-        <v>390</v>
-      </c>
       <c r="I114" s="39" t="s">
         <v>72</v>
       </c>
       <c r="J114" s="39" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="K114" s="39" t="s">
         <v>356</v>
@@ -5398,251 +5837,1107 @@
     </row>
     <row r="115" spans="6:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="F115" s="39" t="s">
+        <v>390</v>
+      </c>
+      <c r="G115" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="H115" s="39" t="s">
         <v>391</v>
       </c>
-      <c r="G115" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="H115" s="39" t="s">
+      <c r="I115" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="L115" s="40" t="s">
         <v>392</v>
-      </c>
-      <c r="I115" s="39" t="s">
-        <v>66</v>
-      </c>
-      <c r="L115" s="40" t="s">
-        <v>393</v>
       </c>
     </row>
     <row r="116" spans="6:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="F116" s="39" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="G116" s="39" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="H116" s="39" t="s">
+        <v>394</v>
+      </c>
+      <c r="I116" s="39" t="s">
+        <v>66</v>
+      </c>
+      <c r="J116" s="39" t="s">
+        <v>393</v>
+      </c>
+      <c r="K116" s="39" t="s">
+        <v>365</v>
+      </c>
+      <c r="L116" s="40" t="s">
         <v>395</v>
       </c>
-      <c r="I116" s="39" t="s">
-        <v>66</v>
-      </c>
-      <c r="J116" s="39" t="s">
-        <v>394</v>
-      </c>
-      <c r="K116" s="39" t="s">
-        <v>366</v>
-      </c>
-      <c r="L116" s="40" t="s">
+    </row>
+    <row r="117" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F117" s="44" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="117" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F117" s="46" t="s">
+      <c r="G117" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H117" s="44" t="s">
+        <v>398</v>
+      </c>
+      <c r="I117" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J117" s="45"/>
+      <c r="K117" s="45"/>
+    </row>
+    <row r="118" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F118" s="44" t="s">
+        <v>399</v>
+      </c>
+      <c r="G118" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H118" s="44" t="s">
+        <v>400</v>
+      </c>
+      <c r="I118" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J118" s="45"/>
+      <c r="K118" s="45"/>
+    </row>
+    <row r="119" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F119" s="44" t="s">
+        <v>401</v>
+      </c>
+      <c r="G119" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H119" s="44" t="s">
+        <v>402</v>
+      </c>
+      <c r="I119" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J119" s="45"/>
+      <c r="K119" s="45"/>
+    </row>
+    <row r="120" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F120" s="44" t="s">
+        <v>403</v>
+      </c>
+      <c r="G120" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H120" s="44" t="s">
+        <v>404</v>
+      </c>
+      <c r="I120" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J120" s="45"/>
+      <c r="K120" s="45"/>
+    </row>
+    <row r="121" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F121" s="44" t="s">
+        <v>405</v>
+      </c>
+      <c r="G121" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H121" s="44" t="s">
+        <v>406</v>
+      </c>
+      <c r="I121" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J121" s="45"/>
+      <c r="K121" s="45"/>
+    </row>
+    <row r="122" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F122" s="44" t="s">
+        <v>407</v>
+      </c>
+      <c r="G122" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H122" s="44" t="s">
+        <v>408</v>
+      </c>
+      <c r="I122" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J122" s="45"/>
+      <c r="K122" s="45"/>
+    </row>
+    <row r="123" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F123" s="44" t="s">
         <v>409</v>
       </c>
-      <c r="G117" s="46" t="s">
+      <c r="G123" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H123" s="44" t="s">
         <v>410</v>
       </c>
-      <c r="H117" s="46" t="s">
+      <c r="I123" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J123" s="45"/>
+      <c r="K123" s="45"/>
+    </row>
+    <row r="124" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F124" s="44" t="s">
         <v>411</v>
       </c>
-      <c r="I117" s="46" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="118" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F118" s="46" t="s">
+      <c r="G124" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H124" s="44" t="s">
         <v>412</v>
       </c>
-      <c r="G118" s="46" t="s">
-        <v>410</v>
-      </c>
-      <c r="H118" s="46" t="s">
+      <c r="I124" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J124" s="45"/>
+      <c r="K124" s="45"/>
+    </row>
+    <row r="125" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F125" s="44" t="s">
         <v>413</v>
       </c>
-      <c r="I118" s="46" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="119" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F119" s="46" t="s">
+      <c r="G125" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H125" s="44" t="s">
         <v>414</v>
       </c>
-      <c r="G119" s="46" t="s">
-        <v>410</v>
-      </c>
-      <c r="H119" s="46" t="s">
+      <c r="I125" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J125" s="45"/>
+      <c r="K125" s="45"/>
+      <c r="L125" s="47" t="s">
         <v>415</v>
       </c>
-      <c r="I119" s="46" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="120" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F120" s="46" t="s">
+    </row>
+    <row r="126" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F126" s="44" t="s">
         <v>416</v>
       </c>
-      <c r="G120" s="46" t="s">
-        <v>410</v>
-      </c>
-      <c r="H120" s="46" t="s">
+      <c r="G126" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H126" s="44" t="s">
         <v>417</v>
       </c>
-      <c r="I120" s="46" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="121" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F121" s="46" t="s">
+      <c r="I126" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J126" s="45"/>
+      <c r="K126" s="45"/>
+      <c r="L126" s="47" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="127" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F127" s="44" t="s">
         <v>418</v>
       </c>
-      <c r="G121" s="46" t="s">
-        <v>410</v>
-      </c>
-      <c r="H121" s="46" t="s">
+      <c r="G127" s="44" t="s">
+        <v>397</v>
+      </c>
+      <c r="H127" s="44" t="s">
         <v>419</v>
       </c>
-      <c r="I121" s="46" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="122" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F122" s="46" t="s">
-        <v>420</v>
-      </c>
-      <c r="G122" s="46" t="s">
-        <v>410</v>
-      </c>
-      <c r="H122" s="46" t="s">
-        <v>421</v>
-      </c>
-      <c r="I122" s="46" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="123" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F123" s="46" t="s">
+      <c r="I127" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J127" s="45"/>
+      <c r="K127" s="45"/>
+      <c r="L127" s="47" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="128" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F128" s="45" t="s">
+        <v>423</v>
+      </c>
+      <c r="G128" s="45" t="s">
         <v>422</v>
       </c>
-      <c r="G123" s="46" t="s">
-        <v>410</v>
-      </c>
-      <c r="H123" s="46" t="s">
-        <v>423</v>
-      </c>
-      <c r="I123" s="46" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="124" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F124" s="46" t="s">
+      <c r="H128" s="45" t="s">
         <v>424</v>
       </c>
-      <c r="G124" s="46" t="s">
-        <v>410</v>
-      </c>
-      <c r="H124" s="46" t="s">
+      <c r="I128" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J128" s="45"/>
+      <c r="K128" s="45"/>
+      <c r="L128" s="47" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="129" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F129" s="45" t="s">
         <v>425</v>
       </c>
-      <c r="I124" s="46" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="125" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F125" s="46" t="s">
+      <c r="G129" s="45" t="s">
+        <v>422</v>
+      </c>
+      <c r="H129" s="45" t="s">
         <v>426</v>
       </c>
-      <c r="G125" s="46" t="s">
-        <v>410</v>
-      </c>
-      <c r="H125" s="46" t="s">
+      <c r="I129" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J129" s="45"/>
+      <c r="K129" s="45"/>
+    </row>
+    <row r="130" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F130" s="45" t="s">
         <v>427</v>
       </c>
-      <c r="I125" s="46" t="s">
-        <v>66</v>
-      </c>
-      <c r="L125" s="47" t="s">
+      <c r="G130" s="45" t="s">
+        <v>422</v>
+      </c>
+      <c r="H130" s="45" t="s">
         <v>428</v>
       </c>
-    </row>
-    <row r="126" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F126" s="46" t="s">
+      <c r="I130" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J130" s="45"/>
+      <c r="K130" s="45"/>
+    </row>
+    <row r="131" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F131" s="45" t="s">
         <v>429</v>
       </c>
-      <c r="G126" s="46" t="s">
-        <v>410</v>
-      </c>
-      <c r="H126" s="46" t="s">
+      <c r="G131" s="45" t="s">
         <v>430</v>
       </c>
-      <c r="I126" s="46" t="s">
-        <v>66</v>
-      </c>
-      <c r="L126" s="47" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="127" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F127" s="46" t="s">
+      <c r="H131" s="45" t="s">
         <v>431</v>
       </c>
-      <c r="G127" s="46" t="s">
-        <v>410</v>
-      </c>
-      <c r="H127" s="46" t="s">
+      <c r="I131" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J131" s="45"/>
+      <c r="K131" s="45"/>
+      <c r="L131" s="47" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="132" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F132" s="45" t="s">
         <v>432</v>
       </c>
-      <c r="I127" s="46" t="s">
-        <v>66</v>
-      </c>
-      <c r="L127" s="47" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="128">
-      <c r="F128" t="s" s="57">
+      <c r="G132" s="45" t="s">
+        <v>430</v>
+      </c>
+      <c r="H132" s="45" t="s">
+        <v>433</v>
+      </c>
+      <c r="I132" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J132" s="45"/>
+      <c r="K132" s="45"/>
+      <c r="L132" s="47" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="133" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F133" s="45" t="s">
+        <v>434</v>
+      </c>
+      <c r="G133" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H133" s="45" t="s">
+        <v>436</v>
+      </c>
+      <c r="I133" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J133" s="45"/>
+      <c r="K133" s="45"/>
+      <c r="L133" s="45"/>
+    </row>
+    <row r="134" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F134" s="45" t="s">
+        <v>437</v>
+      </c>
+      <c r="G134" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H134" s="45" t="s">
+        <v>438</v>
+      </c>
+      <c r="I134" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J134" s="45"/>
+      <c r="K134" s="45"/>
+      <c r="L134" s="45"/>
+    </row>
+    <row r="135" spans="6:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F135" s="45" t="s">
+        <v>439</v>
+      </c>
+      <c r="G135" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H135" s="45" t="s">
+        <v>440</v>
+      </c>
+      <c r="I135" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J135" s="45"/>
+      <c r="K135" s="45"/>
+      <c r="L135" s="47" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="136" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F136" s="45" t="s">
         <v>442</v>
       </c>
-      <c r="G128" t="s" s="57">
-        <v>440</v>
-      </c>
-      <c r="H128" t="s" s="57">
+      <c r="G136" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H136" s="45" t="s">
         <v>443</v>
       </c>
-      <c r="I128" t="s" s="57">
-        <v>66</v>
-      </c>
-      <c r="L128" t="s" s="58">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="F129" t="s" s="59">
+      <c r="I136" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J136" s="45"/>
+      <c r="K136" s="45"/>
+      <c r="L136" s="45"/>
+    </row>
+    <row r="137" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F137" s="45" t="s">
         <v>444</v>
       </c>
-      <c r="G129" t="s" s="59">
-        <v>440</v>
-      </c>
-      <c r="H129" t="s" s="59">
+      <c r="G137" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H137" s="45" t="s">
         <v>445</v>
       </c>
-      <c r="I129" t="s" s="59">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="F130" t="s" s="63">
+      <c r="I137" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J137" s="45"/>
+      <c r="K137" s="45"/>
+      <c r="L137" s="45"/>
+    </row>
+    <row r="138" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F138" s="45" t="s">
+        <v>446</v>
+      </c>
+      <c r="G138" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H138" s="45" t="s">
+        <v>447</v>
+      </c>
+      <c r="I138" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J138" s="45"/>
+      <c r="K138" s="45"/>
+      <c r="L138" s="45"/>
+    </row>
+    <row r="139" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F139" s="45" t="s">
+        <v>448</v>
+      </c>
+      <c r="G139" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H139" s="45" t="s">
+        <v>449</v>
+      </c>
+      <c r="I139" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J139" s="45"/>
+      <c r="K139" s="45"/>
+      <c r="L139" s="45"/>
+    </row>
+    <row r="140" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F140" s="45" t="s">
+        <v>450</v>
+      </c>
+      <c r="G140" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H140" s="45" t="s">
         <v>451</v>
       </c>
-      <c r="G130" t="s" s="63">
-        <v>440</v>
-      </c>
-      <c r="H130" t="s" s="63">
+      <c r="I140" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J140" s="45"/>
+      <c r="K140" s="45"/>
+      <c r="L140" s="45"/>
+    </row>
+    <row r="141" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F141" s="45" t="s">
         <v>452</v>
       </c>
-      <c r="I130" t="s" s="63">
-        <v>72</v>
-      </c>
+      <c r="G141" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H141" s="45" t="s">
+        <v>453</v>
+      </c>
+      <c r="I141" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J141" s="45"/>
+      <c r="K141" s="45"/>
+      <c r="L141" s="45"/>
+    </row>
+    <row r="142" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F142" s="45" t="s">
+        <v>454</v>
+      </c>
+      <c r="G142" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H142" s="45" t="s">
+        <v>455</v>
+      </c>
+      <c r="I142" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J142" s="45"/>
+      <c r="K142" s="45"/>
+      <c r="L142" s="45"/>
+    </row>
+    <row r="143" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F143" s="45" t="s">
+        <v>456</v>
+      </c>
+      <c r="G143" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H143" s="45" t="s">
+        <v>457</v>
+      </c>
+      <c r="I143" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J143" s="45"/>
+      <c r="K143" s="45"/>
+      <c r="L143" s="45"/>
+    </row>
+    <row r="144" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F144" s="45" t="s">
+        <v>458</v>
+      </c>
+      <c r="G144" s="45" t="s">
+        <v>435</v>
+      </c>
+      <c r="H144" s="45" t="s">
+        <v>459</v>
+      </c>
+      <c r="I144" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J144" s="45"/>
+      <c r="K144" s="45"/>
+      <c r="L144" s="45"/>
+    </row>
+    <row r="145" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F145" s="45" t="s">
+        <v>460</v>
+      </c>
+      <c r="G145" s="45" t="s">
+        <v>461</v>
+      </c>
+      <c r="H145" s="45" t="s">
+        <v>462</v>
+      </c>
+      <c r="I145" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J145" s="45"/>
+      <c r="K145" s="45"/>
+      <c r="L145" s="45"/>
+    </row>
+    <row r="146" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F146" s="45" t="s">
+        <v>463</v>
+      </c>
+      <c r="G146" s="45" t="s">
+        <v>461</v>
+      </c>
+      <c r="H146" s="45" t="s">
+        <v>464</v>
+      </c>
+      <c r="I146" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J146" s="45"/>
+      <c r="K146" s="45"/>
+      <c r="L146" s="45"/>
+    </row>
+    <row r="147" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F147" s="45" t="s">
+        <v>465</v>
+      </c>
+      <c r="G147" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H147" s="45" t="s">
+        <v>467</v>
+      </c>
+      <c r="I147" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J147" s="45"/>
+      <c r="K147" s="45"/>
+      <c r="L147" s="47" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="148" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F148" s="45" t="s">
+        <v>468</v>
+      </c>
+      <c r="G148" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H148" s="45" t="s">
+        <v>469</v>
+      </c>
+      <c r="I148" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J148" s="45"/>
+      <c r="K148" s="45"/>
+      <c r="L148" s="47" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="149" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F149" s="45" t="s">
+        <v>470</v>
+      </c>
+      <c r="G149" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H149" s="45" t="s">
+        <v>471</v>
+      </c>
+      <c r="I149" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J149" s="45"/>
+      <c r="K149" s="45"/>
+      <c r="L149" s="47" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="150" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F150" s="45" t="s">
+        <v>472</v>
+      </c>
+      <c r="G150" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H150" s="45" t="s">
+        <v>473</v>
+      </c>
+      <c r="I150" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J150" s="45"/>
+      <c r="K150" s="45"/>
+      <c r="L150" s="47" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="151" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F151" s="45" t="s">
+        <v>474</v>
+      </c>
+      <c r="G151" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H151" s="45" t="s">
+        <v>475</v>
+      </c>
+      <c r="I151" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J151" s="45"/>
+      <c r="K151" s="45"/>
+      <c r="L151" s="47" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="152" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F152" s="45" t="s">
+        <v>476</v>
+      </c>
+      <c r="G152" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H152" s="45" t="s">
+        <v>477</v>
+      </c>
+      <c r="I152" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J152" s="45"/>
+      <c r="K152" s="45"/>
+    </row>
+    <row r="153" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F153" s="45" t="s">
+        <v>478</v>
+      </c>
+      <c r="G153" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H153" s="45" t="s">
+        <v>479</v>
+      </c>
+      <c r="I153" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J153" s="45"/>
+      <c r="K153" s="45"/>
+      <c r="L153" s="47" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="154" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F154" s="45" t="s">
+        <v>481</v>
+      </c>
+      <c r="G154" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H154" s="45" t="s">
+        <v>482</v>
+      </c>
+      <c r="I154" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J154" s="45"/>
+      <c r="K154" s="45"/>
+      <c r="L154" s="45"/>
+    </row>
+    <row r="155" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F155" s="45" t="s">
+        <v>483</v>
+      </c>
+      <c r="G155" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H155" s="45" t="s">
+        <v>484</v>
+      </c>
+      <c r="I155" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J155" s="45"/>
+      <c r="K155" s="45"/>
+      <c r="L155" s="45"/>
+    </row>
+    <row r="156" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F156" s="45" t="s">
+        <v>485</v>
+      </c>
+      <c r="G156" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H156" s="45" t="s">
+        <v>486</v>
+      </c>
+      <c r="I156" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J156" s="45"/>
+      <c r="K156" s="45"/>
+      <c r="L156" s="45"/>
+    </row>
+    <row r="157" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F157" s="45" t="s">
+        <v>487</v>
+      </c>
+      <c r="G157" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H157" s="45" t="s">
+        <v>488</v>
+      </c>
+      <c r="I157" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J157" s="45"/>
+      <c r="K157" s="45"/>
+      <c r="L157" s="45"/>
+    </row>
+    <row r="158" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F158" s="45" t="s">
+        <v>490</v>
+      </c>
+      <c r="G158" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H158" s="45" t="s">
+        <v>491</v>
+      </c>
+      <c r="I158" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J158" s="45"/>
+      <c r="K158" s="45"/>
+      <c r="L158" s="45"/>
+    </row>
+    <row r="159" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F159" s="45" t="s">
+        <v>492</v>
+      </c>
+      <c r="G159" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H159" s="45" t="s">
+        <v>493</v>
+      </c>
+      <c r="I159" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J159" s="45"/>
+      <c r="K159" s="45"/>
+      <c r="L159" s="45"/>
+    </row>
+    <row r="160" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F160" s="45" t="s">
+        <v>494</v>
+      </c>
+      <c r="G160" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H160" s="45" t="s">
+        <v>495</v>
+      </c>
+      <c r="I160" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J160" s="45"/>
+      <c r="K160" s="45"/>
+      <c r="L160" s="45"/>
+    </row>
+    <row r="161" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F161" s="45" t="s">
+        <v>496</v>
+      </c>
+      <c r="G161" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H161" s="45" t="s">
+        <v>497</v>
+      </c>
+      <c r="I161" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J161" s="45"/>
+      <c r="K161" s="45"/>
+      <c r="L161" s="45"/>
+    </row>
+    <row r="162" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F162" s="45" t="s">
+        <v>498</v>
+      </c>
+      <c r="G162" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H162" s="45" t="s">
+        <v>499</v>
+      </c>
+      <c r="I162" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J162" s="45"/>
+      <c r="K162" s="45"/>
+      <c r="L162" s="45"/>
+    </row>
+    <row r="163" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F163" s="45" t="s">
+        <v>503</v>
+      </c>
+      <c r="G163" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H163" s="45" t="s">
+        <v>504</v>
+      </c>
+      <c r="I163" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J163" s="45"/>
+      <c r="K163" s="45"/>
+      <c r="L163" s="45"/>
+    </row>
+    <row r="164" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F164" s="45" t="s">
+        <v>505</v>
+      </c>
+      <c r="G164" s="45" t="s">
+        <v>466</v>
+      </c>
+      <c r="H164" s="45" t="s">
+        <v>506</v>
+      </c>
+      <c r="I164" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="J164" s="45"/>
+      <c r="K164" s="45"/>
+      <c r="L164" s="47" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="165" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F165" s="45" t="s">
+        <v>508</v>
+      </c>
+      <c r="G165" s="45" t="s">
+        <v>509</v>
+      </c>
+      <c r="H165" s="45" t="s">
+        <v>510</v>
+      </c>
+      <c r="I165" s="46" t="s">
+        <v>72</v>
+      </c>
+      <c r="J165" s="45"/>
+      <c r="K165" s="45"/>
+      <c r="L165" s="45"/>
+    </row>
+    <row r="166" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F166" s="48" t="s">
+        <v>512</v>
+      </c>
+      <c r="G166" s="48" t="s">
+        <v>509</v>
+      </c>
+      <c r="H166" s="48" t="s">
+        <v>513</v>
+      </c>
+      <c r="I166" s="48" t="s">
+        <v>72</v>
+      </c>
+      <c r="J166" s="48" t="s">
+        <v>511</v>
+      </c>
+      <c r="K166" s="48" t="s">
+        <v>466</v>
+      </c>
+      <c r="L166" s="45"/>
+    </row>
+    <row r="167" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F167" s="49" t="s">
+        <v>514</v>
+      </c>
+      <c r="G167" s="49" t="s">
+        <v>509</v>
+      </c>
+      <c r="H167" s="49" t="s">
+        <v>515</v>
+      </c>
+      <c r="I167" s="49" t="s">
+        <v>72</v>
+      </c>
+      <c r="J167" s="50">
+        <v>2077089</v>
+      </c>
+      <c r="K167" s="48" t="s">
+        <v>516</v>
+      </c>
+      <c r="L167" s="45"/>
+    </row>
+    <row r="168" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F168" s="51" t="s">
+        <v>517</v>
+      </c>
+      <c r="G168" s="51" t="s">
+        <v>509</v>
+      </c>
+      <c r="H168" s="51" t="s">
+        <v>518</v>
+      </c>
+      <c r="I168" s="51" t="s">
+        <v>72</v>
+      </c>
+      <c r="J168" s="45"/>
+      <c r="K168" s="45"/>
+      <c r="L168" s="45"/>
+    </row>
+    <row r="169" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F169" s="51" t="s">
+        <v>520</v>
+      </c>
+      <c r="G169" s="51" t="s">
+        <v>509</v>
+      </c>
+      <c r="H169" s="51" t="s">
+        <v>521</v>
+      </c>
+      <c r="I169" s="51" t="s">
+        <v>72</v>
+      </c>
+      <c r="J169" s="51" t="s">
+        <v>519</v>
+      </c>
+      <c r="K169" s="51" t="s">
+        <v>509</v>
+      </c>
+      <c r="L169" s="45"/>
+    </row>
+    <row r="170" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F170" s="51" t="s">
+        <v>522</v>
+      </c>
+      <c r="G170" s="51" t="s">
+        <v>523</v>
+      </c>
+      <c r="H170" s="51" t="s">
+        <v>524</v>
+      </c>
+      <c r="I170" s="51" t="s">
+        <v>72</v>
+      </c>
+      <c r="J170" s="51"/>
+      <c r="K170" s="45"/>
+      <c r="L170" s="45"/>
+    </row>
+    <row r="171" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F171" s="52" t="s">
+        <v>525</v>
+      </c>
+      <c r="G171" s="52" t="s">
+        <v>509</v>
+      </c>
+      <c r="H171" s="52" t="s">
+        <v>526</v>
+      </c>
+      <c r="I171" s="52" t="s">
+        <v>72</v>
+      </c>
+      <c r="J171" s="45"/>
+      <c r="K171" s="45"/>
+      <c r="L171" s="45"/>
+    </row>
+    <row r="172" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F172" s="52" t="s">
+        <v>527</v>
+      </c>
+      <c r="G172" s="52" t="s">
+        <v>509</v>
+      </c>
+      <c r="H172" s="52" t="s">
+        <v>528</v>
+      </c>
+      <c r="I172" s="52" t="s">
+        <v>72</v>
+      </c>
+      <c r="J172" s="45"/>
+      <c r="K172" s="45"/>
+      <c r="L172" s="45"/>
+    </row>
+    <row r="173" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F173" s="52" t="s">
+        <v>532</v>
+      </c>
+      <c r="G173" s="52" t="s">
+        <v>533</v>
+      </c>
+      <c r="H173" s="52" t="s">
+        <v>534</v>
+      </c>
+      <c r="I173" s="52" t="s">
+        <v>72</v>
+      </c>
+      <c r="J173" s="45"/>
+      <c r="K173" s="45"/>
+      <c r="L173" s="45"/>
+    </row>
+    <row r="174" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F174" s="52" t="s">
+        <v>536</v>
+      </c>
+      <c r="G174" s="52" t="s">
+        <v>533</v>
+      </c>
+      <c r="H174" s="52" t="s">
+        <v>537</v>
+      </c>
+      <c r="I174" s="52" t="s">
+        <v>72</v>
+      </c>
+      <c r="J174" s="52" t="s">
+        <v>535</v>
+      </c>
+      <c r="K174" s="52" t="s">
+        <v>533</v>
+      </c>
+      <c r="L174" s="45"/>
+    </row>
+    <row r="175" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F175" s="45"/>
+      <c r="G175" s="45"/>
+      <c r="H175" s="45"/>
+      <c r="I175" s="45"/>
+      <c r="J175" s="45"/>
+      <c r="K175" s="45"/>
+      <c r="L175" s="45"/>
+    </row>
+    <row r="176" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F176" s="45"/>
+      <c r="G176" s="45"/>
+      <c r="H176" s="45"/>
+      <c r="I176" s="45"/>
+      <c r="J176" s="45"/>
+      <c r="K176" s="45"/>
+      <c r="L176" s="45"/>
+    </row>
+    <row r="177" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F177" s="45"/>
+      <c r="G177" s="45"/>
+      <c r="H177" s="45"/>
+      <c r="I177" s="45"/>
+      <c r="J177" s="45"/>
+      <c r="K177" s="45"/>
+      <c r="L177" s="45"/>
+    </row>
+    <row r="178" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F178" s="45"/>
+      <c r="G178" s="45"/>
+      <c r="H178" s="45"/>
+      <c r="I178" s="45"/>
+      <c r="J178" s="45"/>
+      <c r="K178" s="45"/>
+      <c r="L178" s="45"/>
+    </row>
+    <row r="179" spans="6:12" x14ac:dyDescent="0.3">
+      <c r="F179" s="45"/>
+      <c r="G179" s="45"/>
+      <c r="H179" s="45"/>
+      <c r="I179" s="45"/>
+      <c r="J179" s="45"/>
+      <c r="K179" s="45"/>
+      <c r="L179" s="45"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -5658,7 +6953,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70924E6C-D075-47E0-B0CB-3BEFA71EC108}">
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="12.77734375"/>
@@ -5671,7 +6966,7 @@
     <col min="8" max="8" bestFit="true" customWidth="true" width="13.6640625"/>
     <col min="9" max="9" bestFit="true" customWidth="true" width="14.88671875"/>
     <col min="10" max="10" bestFit="true" customWidth="true" width="7.88671875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="9.77734375"/>
+    <col min="11" max="11" bestFit="true" customWidth="true" width="10.33203125"/>
     <col min="12" max="12" customWidth="true" width="50.0"/>
   </cols>
   <sheetData>
@@ -5709,6 +7004,9 @@
       <c r="K1" s="42" t="s">
         <v>47</v>
       </c>
+      <c r="L1" s="19" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -5724,26 +7022,27 @@
         <v>39</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="F2" s="41" t="s">
-        <v>64</v>
-      </c>
-      <c r="G2" s="41" t="s">
-        <v>366</v>
-      </c>
-      <c r="H2" s="41" t="s">
-        <v>401</v>
-      </c>
-      <c r="I2" s="41" t="s">
-        <v>72</v>
-      </c>
-      <c r="J2" s="41" t="s">
-        <v>400</v>
-      </c>
-      <c r="K2" s="43" t="s">
-        <v>366</v>
-      </c>
+        <v>420</v>
+      </c>
+      <c r="F2" s="52" t="s">
+        <v>520</v>
+      </c>
+      <c r="G2" s="52" t="s">
+        <v>509</v>
+      </c>
+      <c r="H2" s="52" t="s">
+        <v>521</v>
+      </c>
+      <c r="I2" s="52" t="s">
+        <v>72</v>
+      </c>
+      <c r="J2" s="52" t="s">
+        <v>519</v>
+      </c>
+      <c r="K2" s="52" t="s">
+        <v>509</v>
+      </c>
+      <c r="L2" s="53"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -5759,23 +7058,27 @@
         <v>39</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="F3" s="41" t="s">
-        <v>70</v>
-      </c>
-      <c r="G3" s="41" t="s">
-        <v>366</v>
-      </c>
-      <c r="H3" s="41" t="s">
-        <v>397</v>
-      </c>
-      <c r="I3" s="41" t="s">
-        <v>66</v>
-      </c>
-      <c r="J3" s="41"/>
-      <c r="K3" s="41"/>
-      <c r="L3" s="44"/>
+        <v>421</v>
+      </c>
+      <c r="F3" s="52" t="s">
+        <v>530</v>
+      </c>
+      <c r="G3" s="52" t="s">
+        <v>509</v>
+      </c>
+      <c r="H3" s="52" t="s">
+        <v>531</v>
+      </c>
+      <c r="I3" s="52" t="s">
+        <v>72</v>
+      </c>
+      <c r="J3" s="52" t="s">
+        <v>529</v>
+      </c>
+      <c r="K3" s="52" t="s">
+        <v>509</v>
+      </c>
+      <c r="L3" s="54"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -5791,25 +7094,31 @@
         <v>39</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="F4" s="41" t="s">
-        <v>74</v>
-      </c>
-      <c r="G4" s="41" t="s">
-        <v>366</v>
-      </c>
-      <c r="H4" s="41" t="s">
-        <v>398</v>
-      </c>
-      <c r="I4" s="41" t="s">
-        <v>66</v>
-      </c>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
-      <c r="L4" s="44"/>
+        <v>420</v>
+      </c>
+      <c r="F4" s="52" t="s">
+        <v>536</v>
+      </c>
+      <c r="G4" s="52" t="s">
+        <v>533</v>
+      </c>
+      <c r="H4" s="52" t="s">
+        <v>537</v>
+      </c>
+      <c r="I4" s="52" t="s">
+        <v>72</v>
+      </c>
+      <c r="J4" s="52" t="s">
+        <v>535</v>
+      </c>
+      <c r="K4" s="52" t="s">
+        <v>533</v>
+      </c>
+      <c r="L4" s="54"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A5" s="57"/>
+      <c r="B5" s="57"/>
       <c r="C5" s="2" t="s">
         <v>45</v>
       </c>
@@ -5817,25 +7126,31 @@
         <v>39</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="F5" s="30" t="s">
-        <v>89</v>
-      </c>
-      <c r="G5" s="30" t="s">
-        <v>366</v>
-      </c>
-      <c r="H5" s="30" t="s">
-        <v>399</v>
-      </c>
-      <c r="I5" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="J5" s="41"/>
-      <c r="K5" s="41"/>
-      <c r="L5" s="44"/>
+        <v>421</v>
+      </c>
+      <c r="F5" s="53" t="s">
+        <v>539</v>
+      </c>
+      <c r="G5" s="53" t="s">
+        <v>533</v>
+      </c>
+      <c r="H5" s="53" t="s">
+        <v>540</v>
+      </c>
+      <c r="I5" s="53" t="s">
+        <v>72</v>
+      </c>
+      <c r="J5" s="53" t="s">
+        <v>538</v>
+      </c>
+      <c r="K5" s="53" t="s">
+        <v>533</v>
+      </c>
+      <c r="L5" s="54"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A6" s="57"/>
+      <c r="B6" s="57"/>
       <c r="C6" s="2" t="s">
         <v>45</v>
       </c>
@@ -5843,28 +7158,31 @@
         <v>39</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>433</v>
-      </c>
-      <c r="F6" s="45" t="s">
-        <v>89</v>
-      </c>
-      <c r="G6" s="45" t="s">
-        <v>366</v>
-      </c>
-      <c r="H6" s="45" t="s">
-        <v>403</v>
-      </c>
-      <c r="I6" s="45" t="s">
-        <v>72</v>
-      </c>
-      <c r="J6" s="45" t="s">
-        <v>402</v>
-      </c>
-      <c r="K6" s="45" t="s">
-        <v>366</v>
-      </c>
+        <v>420</v>
+      </c>
+      <c r="F6" s="55" t="s">
+        <v>542</v>
+      </c>
+      <c r="G6" s="55" t="s">
+        <v>533</v>
+      </c>
+      <c r="H6" s="55" t="s">
+        <v>543</v>
+      </c>
+      <c r="I6" s="55" t="s">
+        <v>72</v>
+      </c>
+      <c r="J6" s="55" t="s">
+        <v>541</v>
+      </c>
+      <c r="K6" s="55" t="s">
+        <v>533</v>
+      </c>
+      <c r="L6" s="53"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A7" s="57"/>
+      <c r="B7" s="57"/>
       <c r="C7" s="2" t="s">
         <v>45</v>
       </c>
@@ -5872,28 +7190,29 @@
         <v>39</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>434</v>
-      </c>
-      <c r="F7" s="45" t="s">
-        <v>92</v>
-      </c>
-      <c r="G7" s="45" t="s">
-        <v>366</v>
-      </c>
-      <c r="H7" s="45" t="s">
-        <v>408</v>
-      </c>
-      <c r="I7" s="45" t="s">
-        <v>72</v>
-      </c>
-      <c r="J7" s="45" t="s">
-        <v>407</v>
-      </c>
-      <c r="K7" s="45" t="s">
-        <v>366</v>
+        <v>421</v>
+      </c>
+      <c r="F7" s="57" t="s">
+        <v>544</v>
+      </c>
+      <c r="G7" s="57" t="s">
+        <v>533</v>
+      </c>
+      <c r="H7" s="57" t="s">
+        <v>545</v>
+      </c>
+      <c r="I7" s="57" t="s">
+        <v>66</v>
+      </c>
+      <c r="J7" s="43"/>
+      <c r="K7" s="43"/>
+      <c r="L7" s="58" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A8" s="57"/>
+      <c r="B8" s="57"/>
       <c r="C8" s="2" t="s">
         <v>45</v>
       </c>
@@ -5901,26 +7220,27 @@
         <v>39</v>
       </c>
       <c r="E8" s="1"/>
-      <c r="F8" s="56" t="s">
-        <v>95</v>
-      </c>
-      <c r="G8" s="56" t="s">
-        <v>440</v>
-      </c>
-      <c r="H8" s="56" t="s">
-        <v>441</v>
-      </c>
-      <c r="I8" s="56" t="s">
-        <v>72</v>
-      </c>
-      <c r="J8" s="55" t="s">
-        <v>439</v>
-      </c>
-      <c r="K8" s="55" t="s">
-        <v>440</v>
+      <c r="F8" s="57" t="s">
+        <v>546</v>
+      </c>
+      <c r="G8" s="57" t="s">
+        <v>533</v>
+      </c>
+      <c r="H8" s="57" t="s">
+        <v>547</v>
+      </c>
+      <c r="I8" s="57" t="s">
+        <v>66</v>
+      </c>
+      <c r="J8" s="45"/>
+      <c r="K8" s="45"/>
+      <c r="L8" s="58" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A9" s="57"/>
+      <c r="B9" s="57"/>
       <c r="C9" s="2" t="s">
         <v>45</v>
       </c>
@@ -5928,26 +7248,27 @@
         <v>39</v>
       </c>
       <c r="E9" s="1"/>
-      <c r="F9" s="62" t="s">
-        <v>98</v>
-      </c>
-      <c r="G9" s="62" t="s">
-        <v>440</v>
-      </c>
-      <c r="H9" s="62" t="s">
-        <v>450</v>
-      </c>
-      <c r="I9" s="62" t="s">
-        <v>72</v>
-      </c>
-      <c r="J9" s="61" t="s">
-        <v>449</v>
-      </c>
-      <c r="K9" s="61" t="s">
-        <v>440</v>
+      <c r="F9" s="66" t="s">
+        <v>549</v>
+      </c>
+      <c r="G9" s="66" t="s">
+        <v>533</v>
+      </c>
+      <c r="H9" s="66" t="s">
+        <v>550</v>
+      </c>
+      <c r="I9" s="66" t="s">
+        <v>66</v>
+      </c>
+      <c r="J9" s="45"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="67" t="s">
+        <v>548</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A10" s="57"/>
+      <c r="B10" s="57"/>
       <c r="C10" s="2" t="s">
         <v>45</v>
       </c>
@@ -5961,8 +7282,11 @@
       <c r="I10" s="41"/>
       <c r="J10" s="41"/>
       <c r="K10" s="41"/>
+      <c r="L10" s="53"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A11" s="57"/>
+      <c r="B11" s="57"/>
       <c r="C11" s="2" t="s">
         <v>45</v>
       </c>
@@ -5976,8 +7300,11 @@
       <c r="I11" s="41"/>
       <c r="J11" s="41"/>
       <c r="K11" s="41"/>
+      <c r="L11" s="53"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A12" s="57"/>
+      <c r="B12" s="57"/>
       <c r="C12" s="2" t="s">
         <v>45</v>
       </c>
@@ -5991,8 +7318,11 @@
       <c r="I12" s="41"/>
       <c r="J12" s="41"/>
       <c r="K12" s="41"/>
+      <c r="L12" s="53"/>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A13" s="57"/>
+      <c r="B13" s="57"/>
       <c r="C13" s="2" t="s">
         <v>45</v>
       </c>
@@ -6006,8 +7336,11 @@
       <c r="I13" s="41"/>
       <c r="J13" s="41"/>
       <c r="K13" s="41"/>
+      <c r="L13" s="53"/>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A14" s="57"/>
+      <c r="B14" s="57"/>
       <c r="C14" s="2" t="s">
         <v>45</v>
       </c>
@@ -6021,8 +7354,11 @@
       <c r="I14" s="41"/>
       <c r="J14" s="41"/>
       <c r="K14" s="41"/>
+      <c r="L14" s="53"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A15" s="57"/>
+      <c r="B15" s="57"/>
       <c r="C15" s="2" t="s">
         <v>45</v>
       </c>
@@ -6036,23 +7372,247 @@
       <c r="I15" s="41"/>
       <c r="J15" s="41"/>
       <c r="K15" s="41"/>
+      <c r="L15" s="53"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="C16" s="2" t="s">
+      <c r="A16" s="57"/>
+      <c r="B16" s="57"/>
+      <c r="C16" s="65" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="E16" s="1"/>
+      <c r="E16" s="30"/>
       <c r="F16" s="41"/>
       <c r="G16" s="41"/>
       <c r="H16" s="41"/>
       <c r="I16" s="41"/>
       <c r="J16" s="41"/>
       <c r="K16" s="41"/>
+      <c r="L16" s="53"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17" s="57"/>
+      <c r="B17" s="57"/>
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="57"/>
+      <c r="F17" s="55"/>
+      <c r="G17" s="55"/>
+      <c r="H17" s="55"/>
+      <c r="I17" s="55"/>
+      <c r="J17" s="57"/>
+      <c r="K17" s="57"/>
+      <c r="L17" s="56"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18" s="57"/>
+      <c r="B18" s="57"/>
+      <c r="C18" s="57"/>
+      <c r="D18" s="57"/>
+      <c r="E18" s="57"/>
+      <c r="F18" s="57"/>
+      <c r="G18" s="57"/>
+      <c r="H18" s="57"/>
+      <c r="I18" s="57"/>
+      <c r="J18" s="57"/>
+      <c r="K18" s="57"/>
+      <c r="L18" s="57"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19" s="57"/>
+      <c r="B19" s="57"/>
+      <c r="C19" s="57"/>
+      <c r="D19" s="57"/>
+      <c r="E19" s="57"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="57"/>
+      <c r="I19" s="57"/>
+      <c r="J19" s="57"/>
+      <c r="K19" s="57"/>
+      <c r="L19" s="57"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20" s="57"/>
+      <c r="B20" s="57"/>
+      <c r="C20" s="57"/>
+      <c r="D20" s="57"/>
+      <c r="E20" s="57"/>
+      <c r="F20" s="57"/>
+      <c r="G20" s="57"/>
+      <c r="H20" s="57"/>
+      <c r="I20" s="57"/>
+      <c r="J20" s="57"/>
+      <c r="K20" s="57"/>
+      <c r="L20" s="57"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A21" s="57"/>
+      <c r="B21" s="57"/>
+      <c r="C21" s="57"/>
+      <c r="D21" s="57"/>
+      <c r="E21" s="57"/>
+      <c r="F21" s="57"/>
+      <c r="G21" s="57"/>
+      <c r="H21" s="57"/>
+      <c r="I21" s="57"/>
+      <c r="J21" s="57"/>
+      <c r="K21" s="57"/>
+      <c r="L21" s="57"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A22" s="57"/>
+      <c r="B22" s="57"/>
+      <c r="C22" s="57"/>
+      <c r="D22" s="57"/>
+      <c r="E22" s="57"/>
+      <c r="F22" s="57"/>
+      <c r="G22" s="57"/>
+      <c r="H22" s="57"/>
+      <c r="I22" s="57"/>
+      <c r="J22" s="57"/>
+      <c r="K22" s="57"/>
+      <c r="L22" s="57"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A23" s="57"/>
+      <c r="B23" s="57"/>
+      <c r="C23" s="57"/>
+      <c r="D23" s="57"/>
+      <c r="E23" s="57"/>
+      <c r="F23" s="57"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="57"/>
+      <c r="I23" s="57"/>
+      <c r="J23" s="57"/>
+      <c r="K23" s="57"/>
+      <c r="L23" s="57"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A24" s="57"/>
+      <c r="B24" s="57"/>
+      <c r="C24" s="57"/>
+      <c r="D24" s="57"/>
+      <c r="E24" s="57"/>
+      <c r="F24" s="57"/>
+      <c r="G24" s="57"/>
+      <c r="H24" s="57"/>
+      <c r="I24" s="57"/>
+      <c r="J24" s="57"/>
+      <c r="K24" s="57"/>
+      <c r="L24" s="57"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A25" s="57"/>
+      <c r="B25" s="57"/>
+      <c r="C25" s="57"/>
+      <c r="D25" s="57"/>
+      <c r="E25" s="57"/>
+      <c r="F25" s="57"/>
+      <c r="G25" s="57"/>
+      <c r="H25" s="57"/>
+      <c r="I25" s="57"/>
+      <c r="J25" s="57"/>
+      <c r="K25" s="57"/>
+      <c r="L25" s="57"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A26" s="57"/>
+      <c r="B26" s="57"/>
+      <c r="C26" s="57"/>
+      <c r="D26" s="57"/>
+      <c r="E26" s="57"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="57"/>
+      <c r="H26" s="57"/>
+      <c r="I26" s="57"/>
+      <c r="J26" s="57"/>
+      <c r="K26" s="57"/>
+      <c r="L26" s="57"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A27" s="57"/>
+      <c r="B27" s="57"/>
+      <c r="C27" s="57"/>
+      <c r="D27" s="57"/>
+      <c r="E27" s="57"/>
+      <c r="F27" s="57"/>
+      <c r="G27" s="57"/>
+      <c r="H27" s="57"/>
+      <c r="I27" s="57"/>
+      <c r="J27" s="57"/>
+      <c r="K27" s="57"/>
+      <c r="L27" s="57"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A28" s="57"/>
+      <c r="B28" s="57"/>
+      <c r="C28" s="57"/>
+      <c r="D28" s="57"/>
+      <c r="E28" s="57"/>
+      <c r="F28" s="57"/>
+      <c r="G28" s="57"/>
+      <c r="H28" s="57"/>
+      <c r="I28" s="57"/>
+      <c r="J28" s="57"/>
+      <c r="K28" s="57"/>
+      <c r="L28" s="57"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A29" s="57"/>
+      <c r="B29" s="57"/>
+      <c r="C29" s="57"/>
+      <c r="D29" s="57"/>
+      <c r="E29" s="57"/>
+      <c r="F29" s="57"/>
+      <c r="G29" s="57"/>
+      <c r="H29" s="57"/>
+      <c r="I29" s="57"/>
+      <c r="J29" s="57"/>
+      <c r="K29" s="57"/>
+      <c r="L29" s="57"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A30" s="57"/>
+      <c r="B30" s="57"/>
+      <c r="C30" s="57"/>
+      <c r="D30" s="57"/>
+      <c r="E30" s="57"/>
+      <c r="F30" s="57"/>
+      <c r="G30" s="57"/>
+      <c r="H30" s="57"/>
+      <c r="I30" s="57"/>
+      <c r="J30" s="57"/>
+      <c r="K30" s="57"/>
+      <c r="L30" s="57"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A31" s="57"/>
+      <c r="B31" s="57"/>
+      <c r="C31" s="57"/>
+      <c r="D31" s="57"/>
+      <c r="E31" s="57"/>
+      <c r="F31" s="57"/>
+      <c r="G31" s="57"/>
+      <c r="H31" s="57"/>
+      <c r="I31" s="57"/>
+      <c r="J31" s="57"/>
+      <c r="K31" s="57"/>
+      <c r="L31" s="57"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="F32" s="57"/>
+      <c r="G32" s="57"/>
+      <c r="H32" s="57"/>
+      <c r="I32" s="57"/>
+      <c r="J32" s="57"/>
+      <c r="K32" s="57"/>
+      <c r="L32" s="57"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Email sender issues fixed Config file updated Email logo added
</commit_message>
<xml_diff>
--- a/src/test/resources/POC_data_sheet_v1.1.xlsx
+++ b/src/test/resources/POC_data_sheet_v1.1.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1152" uniqueCount="551">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1242" uniqueCount="597">
   <si>
     <t>Application</t>
   </si>
@@ -1695,6 +1695,144 @@
   </si>
   <si>
     <t>13:04:03</t>
+  </si>
+  <si>
+    <t>R173</t>
+  </si>
+  <si>
+    <t>08/14/2025</t>
+  </si>
+  <si>
+    <t>17:33:28</t>
+  </si>
+  <si>
+    <t>R174</t>
+  </si>
+  <si>
+    <t>17:34:50</t>
+  </si>
+  <si>
+    <t>R175</t>
+  </si>
+  <si>
+    <t>19:25:47</t>
+  </si>
+  <si>
+    <t>R176</t>
+  </si>
+  <si>
+    <t>19:26:30</t>
+  </si>
+  <si>
+    <t>R177</t>
+  </si>
+  <si>
+    <t>20:10:54</t>
+  </si>
+  <si>
+    <t>R178</t>
+  </si>
+  <si>
+    <t>20:11:15</t>
+  </si>
+  <si>
+    <t>R179</t>
+  </si>
+  <si>
+    <t>20:13:31</t>
+  </si>
+  <si>
+    <t>R180</t>
+  </si>
+  <si>
+    <t>20:13:53</t>
+  </si>
+  <si>
+    <t>R181</t>
+  </si>
+  <si>
+    <t>20:51:10</t>
+  </si>
+  <si>
+    <t>R182</t>
+  </si>
+  <si>
+    <t>20:51:30</t>
+  </si>
+  <si>
+    <t>R183</t>
+  </si>
+  <si>
+    <t>08/15/2025</t>
+  </si>
+  <si>
+    <t>10:06:14</t>
+  </si>
+  <si>
+    <t>Login was not successful for user: rahul.reddy917@outlook.com</t>
+  </si>
+  <si>
+    <t>R184</t>
+  </si>
+  <si>
+    <t>10:07:26</t>
+  </si>
+  <si>
+    <t>R185</t>
+  </si>
+  <si>
+    <t>10:59:53</t>
+  </si>
+  <si>
+    <t>R186</t>
+  </si>
+  <si>
+    <t>R187</t>
+  </si>
+  <si>
+    <t>11:25:29</t>
+  </si>
+  <si>
+    <t>R188</t>
+  </si>
+  <si>
+    <t>11:26:07</t>
+  </si>
+  <si>
+    <t>R189</t>
+  </si>
+  <si>
+    <t>11:27:50</t>
+  </si>
+  <si>
+    <t>R190</t>
+  </si>
+  <si>
+    <t>11:28:28</t>
+  </si>
+  <si>
+    <t>R191</t>
+  </si>
+  <si>
+    <t>11:50:10</t>
+  </si>
+  <si>
+    <t>R192</t>
+  </si>
+  <si>
+    <t>11:50:31</t>
+  </si>
+  <si>
+    <t>R193</t>
+  </si>
+  <si>
+    <t>12:00:15</t>
+  </si>
+  <si>
+    <t>R194</t>
+  </si>
+  <si>
+    <t>12:00:36</t>
   </si>
 </sst>
 </file>
@@ -2165,7 +2303,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2320,6 +2458,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true">
       <alignment wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="true"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3049,7 +3215,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{087D34EC-64B6-464A-B1FA-1B3B12C5A42D}">
-  <dimension ref="A1:L179"/>
+  <dimension ref="A1:L196"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="15.44140625"/>
@@ -6895,49 +7061,333 @@
       <c r="L174" s="45"/>
     </row>
     <row r="175" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F175" s="45"/>
-      <c r="G175" s="45"/>
-      <c r="H175" s="45"/>
-      <c r="I175" s="45"/>
+      <c r="F175" s="68" t="s">
+        <v>551</v>
+      </c>
+      <c r="G175" s="68" t="s">
+        <v>552</v>
+      </c>
+      <c r="H175" s="68" t="s">
+        <v>553</v>
+      </c>
+      <c r="I175" s="68" t="s">
+        <v>72</v>
+      </c>
       <c r="J175" s="45"/>
       <c r="K175" s="45"/>
       <c r="L175" s="45"/>
     </row>
     <row r="176" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F176" s="45"/>
-      <c r="G176" s="45"/>
-      <c r="H176" s="45"/>
-      <c r="I176" s="45"/>
+      <c r="F176" s="69" t="s">
+        <v>554</v>
+      </c>
+      <c r="G176" s="69" t="s">
+        <v>552</v>
+      </c>
+      <c r="H176" s="69" t="s">
+        <v>555</v>
+      </c>
+      <c r="I176" s="69" t="s">
+        <v>72</v>
+      </c>
       <c r="J176" s="45"/>
       <c r="K176" s="45"/>
       <c r="L176" s="45"/>
     </row>
     <row r="177" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F177" s="45"/>
-      <c r="G177" s="45"/>
-      <c r="H177" s="45"/>
-      <c r="I177" s="45"/>
+      <c r="F177" s="70" t="s">
+        <v>556</v>
+      </c>
+      <c r="G177" s="70" t="s">
+        <v>552</v>
+      </c>
+      <c r="H177" s="70" t="s">
+        <v>557</v>
+      </c>
+      <c r="I177" s="70" t="s">
+        <v>72</v>
+      </c>
       <c r="J177" s="45"/>
       <c r="K177" s="45"/>
       <c r="L177" s="45"/>
     </row>
     <row r="178" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F178" s="45"/>
-      <c r="G178" s="45"/>
-      <c r="H178" s="45"/>
-      <c r="I178" s="45"/>
+      <c r="F178" s="71" t="s">
+        <v>558</v>
+      </c>
+      <c r="G178" s="71" t="s">
+        <v>552</v>
+      </c>
+      <c r="H178" s="71" t="s">
+        <v>559</v>
+      </c>
+      <c r="I178" s="71" t="s">
+        <v>72</v>
+      </c>
       <c r="J178" s="45"/>
       <c r="K178" s="45"/>
       <c r="L178" s="45"/>
     </row>
     <row r="179" spans="6:12" x14ac:dyDescent="0.3">
-      <c r="F179" s="45"/>
-      <c r="G179" s="45"/>
-      <c r="H179" s="45"/>
-      <c r="I179" s="45"/>
+      <c r="F179" s="72" t="s">
+        <v>560</v>
+      </c>
+      <c r="G179" s="72" t="s">
+        <v>552</v>
+      </c>
+      <c r="H179" s="72" t="s">
+        <v>561</v>
+      </c>
+      <c r="I179" s="72" t="s">
+        <v>72</v>
+      </c>
       <c r="J179" s="45"/>
       <c r="K179" s="45"/>
       <c r="L179" s="45"/>
+    </row>
+    <row r="180">
+      <c r="F180" t="s" s="73">
+        <v>562</v>
+      </c>
+      <c r="G180" t="s" s="73">
+        <v>552</v>
+      </c>
+      <c r="H180" t="s" s="73">
+        <v>563</v>
+      </c>
+      <c r="I180" t="s" s="73">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="F181" t="s" s="74">
+        <v>564</v>
+      </c>
+      <c r="G181" t="s" s="74">
+        <v>552</v>
+      </c>
+      <c r="H181" t="s" s="74">
+        <v>565</v>
+      </c>
+      <c r="I181" t="s" s="74">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="F182" t="s" s="75">
+        <v>566</v>
+      </c>
+      <c r="G182" t="s" s="75">
+        <v>552</v>
+      </c>
+      <c r="H182" t="s" s="75">
+        <v>567</v>
+      </c>
+      <c r="I182" t="s" s="75">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="F183" t="s" s="76">
+        <v>568</v>
+      </c>
+      <c r="G183" t="s" s="76">
+        <v>552</v>
+      </c>
+      <c r="H183" t="s" s="76">
+        <v>569</v>
+      </c>
+      <c r="I183" t="s" s="76">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="F184" t="s" s="77">
+        <v>570</v>
+      </c>
+      <c r="G184" t="s" s="77">
+        <v>552</v>
+      </c>
+      <c r="H184" t="s" s="77">
+        <v>571</v>
+      </c>
+      <c r="I184" t="s" s="77">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="F185" t="s" s="78">
+        <v>572</v>
+      </c>
+      <c r="G185" t="s" s="78">
+        <v>573</v>
+      </c>
+      <c r="H185" t="s" s="78">
+        <v>574</v>
+      </c>
+      <c r="I185" t="s" s="78">
+        <v>66</v>
+      </c>
+      <c r="L185" t="s" s="79">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="F186" t="s" s="80">
+        <v>576</v>
+      </c>
+      <c r="G186" t="s" s="80">
+        <v>573</v>
+      </c>
+      <c r="H186" t="s" s="80">
+        <v>577</v>
+      </c>
+      <c r="I186" t="s" s="80">
+        <v>66</v>
+      </c>
+      <c r="L186" t="s" s="81">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="F187" t="s" s="82">
+        <v>578</v>
+      </c>
+      <c r="G187" t="s" s="82">
+        <v>573</v>
+      </c>
+      <c r="H187" t="s" s="82">
+        <v>579</v>
+      </c>
+      <c r="I187" t="s" s="82">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="F188" t="s" s="83">
+        <v>580</v>
+      </c>
+      <c r="G188" t="s" s="83">
+        <v>573</v>
+      </c>
+      <c r="H188" t="s" s="83">
+        <v>158</v>
+      </c>
+      <c r="I188" t="s" s="83">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="F189" t="s" s="84">
+        <v>581</v>
+      </c>
+      <c r="G189" t="s" s="84">
+        <v>573</v>
+      </c>
+      <c r="H189" t="s" s="84">
+        <v>582</v>
+      </c>
+      <c r="I189" t="s" s="84">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="F190" t="s" s="85">
+        <v>583</v>
+      </c>
+      <c r="G190" t="s" s="85">
+        <v>573</v>
+      </c>
+      <c r="H190" t="s" s="85">
+        <v>584</v>
+      </c>
+      <c r="I190" t="s" s="85">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="F191" t="s" s="86">
+        <v>585</v>
+      </c>
+      <c r="G191" t="s" s="86">
+        <v>573</v>
+      </c>
+      <c r="H191" t="s" s="86">
+        <v>586</v>
+      </c>
+      <c r="I191" t="s" s="86">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="F192" t="s" s="87">
+        <v>587</v>
+      </c>
+      <c r="G192" t="s" s="87">
+        <v>573</v>
+      </c>
+      <c r="H192" t="s" s="87">
+        <v>588</v>
+      </c>
+      <c r="I192" t="s" s="87">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="F193" t="s" s="88">
+        <v>589</v>
+      </c>
+      <c r="G193" t="s" s="88">
+        <v>573</v>
+      </c>
+      <c r="H193" t="s" s="88">
+        <v>590</v>
+      </c>
+      <c r="I193" t="s" s="88">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="F194" t="s" s="89">
+        <v>591</v>
+      </c>
+      <c r="G194" t="s" s="89">
+        <v>573</v>
+      </c>
+      <c r="H194" t="s" s="89">
+        <v>592</v>
+      </c>
+      <c r="I194" t="s" s="89">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="F195" t="s" s="90">
+        <v>593</v>
+      </c>
+      <c r="G195" t="s" s="90">
+        <v>573</v>
+      </c>
+      <c r="H195" t="s" s="90">
+        <v>594</v>
+      </c>
+      <c r="I195" t="s" s="90">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="F196" t="s" s="91">
+        <v>595</v>
+      </c>
+      <c r="G196" t="s" s="91">
+        <v>573</v>
+      </c>
+      <c r="H196" t="s" s="91">
+        <v>596</v>
+      </c>
+      <c r="I196" t="s" s="91">
+        <v>72</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>